<commit_message>
feat: Add Expense and Income pages with transaction management
- Implemented ExpensePage component for tracking expenses, including adding, editing, and deleting transactions.
- Created Income component for managing income sources with similar functionalities.
- Added Profile page as a placeholder for user profile management.
- Introduced exportUtils for exporting transaction data to Excel format.
- Integrated charts for visualizing income and expense trends using recharts.
- Enhanced transaction filtering and overview fetching for both income and expense pages.
</commit_message>
<xml_diff>
--- a/backend/expense_details.xlsx
+++ b/backend/expense_details.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,21 +415,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>fast food</v>
+        <v>sport</v>
       </c>
       <c r="B2">
-        <v>1006</v>
+        <v>1500</v>
       </c>
       <c r="C2" t="str">
-        <v>Fooood</v>
+        <v>Bonus</v>
       </c>
       <c r="D2" t="str">
-        <v>10/6/2026</v>
+        <v>30/6/2026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>fitness food</v>
+        <v>fast food</v>
       </c>
       <c r="B3">
         <v>1006</v>
@@ -438,12 +438,26 @@
         <v>Fooood</v>
       </c>
       <c r="D3" t="str">
+        <v>10/6/2026</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>fitness food</v>
+      </c>
+      <c r="B4">
+        <v>1006</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Fooood</v>
+      </c>
+      <c r="D4" t="str">
         <v>10/6/2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>